<commit_message>
Attendance reports: Excel downloads (monthly, daily, leave card, summary), analytics and company settings
Employees choose At Office / Work From Home / On Duty at punch-in; leave can be
full day, half day or comp-off. One classify_day rule gives every person-day a
code (At Office, WFH, OD, WOW, HW, C/Off, W/Off, Holiday, FD/HD Leave, Absent)
used by the .xlsx exports, the analytics API and the screens.

Owner or a manager holding the new download_company_reports permission can use
the company-wide reports (read-only, audited). Owner manages weekly off, late
time and holidays. New screens: Attendance analytics, Company settings.

Migration 0020. Backend 245 tests, frontend 381, authz sweep 276, real-stack
reports check 33.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/uat/UAT-scenarios.xlsx
+++ b/docs/uat/UAT-scenarios.xlsx
@@ -13,14 +13,16 @@
     <sheet name="Owner" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Manager" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Employee" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Cross-cutting" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Defects" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="HR reports and Excel downloads" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Cross-cutting" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Defects" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Owner'!$A$1:$L$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Manager'!$A$1:$L$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Employee'!$A$1:$L$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Cross-cutting'!$A$1:$L$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'HR reports and Excel downloads'!$A$1:$L$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Cross-cutting'!$A$1:$L$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -620,7 +622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -780,26 +782,26 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cross-cutting</t>
+          <t>HR reports and Excel downloads</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>33</v>
+        <v>7</v>
       </c>
       <c r="C5">
-        <f>COUNTIF('Cross-cutting'!I2:I34,"Pass")</f>
+        <f>COUNTIF('HR reports and Excel downloads'!I2:I8,"Pass")</f>
         <v/>
       </c>
       <c r="D5">
-        <f>COUNTIF('Cross-cutting'!I2:I34,"Fail")</f>
+        <f>COUNTIF('HR reports and Excel downloads'!I2:I8,"Fail")</f>
         <v/>
       </c>
       <c r="E5">
-        <f>COUNTIF('Cross-cutting'!I2:I34,"Blocked")</f>
+        <f>COUNTIF('HR reports and Excel downloads'!I2:I8,"Blocked")</f>
         <v/>
       </c>
       <c r="F5">
-        <f>COUNTIF('Cross-cutting'!I2:I34,"N/A")</f>
+        <f>COUNTIF('HR reports and Excel downloads'!I2:I8,"N/A")</f>
         <v/>
       </c>
       <c r="G5">
@@ -812,33 +814,32 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B6" s="5">
-        <f>SUM(B2:B5)</f>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cross-cutting</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>33</v>
+      </c>
+      <c r="C6">
+        <f>COUNTIF('Cross-cutting'!I2:I34,"Pass")</f>
         <v/>
       </c>
-      <c r="C6" s="5">
-        <f>SUM(C2:C5)</f>
+      <c r="D6">
+        <f>COUNTIF('Cross-cutting'!I2:I34,"Fail")</f>
         <v/>
       </c>
-      <c r="D6" s="5">
-        <f>SUM(D2:D5)</f>
+      <c r="E6">
+        <f>COUNTIF('Cross-cutting'!I2:I34,"Blocked")</f>
         <v/>
       </c>
-      <c r="E6" s="5">
-        <f>SUM(E2:E5)</f>
+      <c r="F6">
+        <f>COUNTIF('Cross-cutting'!I2:I34,"N/A")</f>
         <v/>
       </c>
-      <c r="F6" s="5">
-        <f>SUM(F2:F5)</f>
-        <v/>
-      </c>
-      <c r="G6" s="5">
-        <f>SUM(G2:G5)</f>
+      <c r="G6">
+        <f>B6-SUM(C6:F6)</f>
         <v/>
       </c>
       <c r="H6" s="4">
@@ -846,57 +847,81 @@
         <v/>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B7" s="5">
+        <f>SUM(B2:B6)</f>
+        <v/>
+      </c>
+      <c r="C7" s="5">
+        <f>SUM(C2:C6)</f>
+        <v/>
+      </c>
+      <c r="D7" s="5">
+        <f>SUM(D2:D6)</f>
+        <v/>
+      </c>
+      <c r="E7" s="5">
+        <f>SUM(E2:E6)</f>
+        <v/>
+      </c>
+      <c r="F7" s="5">
+        <f>SUM(F2:F6)</f>
+        <v/>
+      </c>
+      <c r="G7" s="5">
+        <f>SUM(G2:G6)</f>
+        <v/>
+      </c>
+      <c r="H7" s="4">
+        <f>IF(B7=0,0,SUM(C7:F7)/B7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Open blockers</t>
         </is>
       </c>
-      <c r="B8">
+      <c r="B9">
         <f>COUNTIFS(Defects!C2:C200,"Blocker",Defects!H2:H200,"Open")</f>
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Open majors</t>
         </is>
       </c>
-      <c r="B9">
+      <c r="B10">
         <f>COUNTIFS(Defects!C2:C200,"Major",Defects!H2:H200,"Open")</f>
         <v/>
       </c>
     </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Exit criteria (agree before starting): no open Blocker, no open Major without an agreed workaround, every scenario run (Pass, or Fail with a defect, or N/A with a reason).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Sign-off</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Accepted / not accepted</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="8" t="n"/>
-      <c r="D14" s="8" t="n"/>
-      <c r="E14" s="9" t="n"/>
+          <t>Sign-off</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Accepted / not accepted</t>
         </is>
       </c>
       <c r="B15" s="7" t="n"/>
@@ -907,7 +932,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="B16" s="7" t="n"/>
@@ -918,7 +943,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="B17" s="7" t="n"/>
@@ -929,7 +954,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Signature</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B18" s="7" t="n"/>
@@ -937,14 +962,25 @@
       <c r="D18" s="8" t="n"/>
       <c r="E18" s="9" t="n"/>
     </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Signature</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="8" t="n"/>
+      <c r="E19" s="9" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A12:H12"/>
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="B18:E18"/>
     <mergeCell ref="B16:E16"/>
     <mergeCell ref="B15:E15"/>
-    <mergeCell ref="A11:H11"/>
-    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B19:E19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1505,7 +1541,7 @@
         <is>
           <t>- Right after sign-in you are taken to the change-password page and cannot open anything else (typing /tasks in the address bar returns here).
 - A weak password such as "password123" or one containing "OWN001" is refused with a clear message.
-- After a valid change you land on "Company overview" and the menu shows: Company overview, Company tasks, Attendance, Leave requests, EOD reports, Projects, Team calendar, Service calls, Customers, Machines, Reports, Users &amp; hierarchy, Permissions, Audit trail.</t>
+- After a valid change you land on "Company overview" and the menu shows: Company overview, Company tasks, Attendance, Leave requests, EOD reports, Projects, Team calendar, Service calls, Customers, Machines, Reports, Attendance analytics, Users &amp; hierarchy, Permissions, Company settings, Audit trail.</t>
         </is>
       </c>
       <c r="H2" s="10" t="inlineStr"/>
@@ -4990,6 +5026,398 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Expected result</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Actual result</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Tester</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>UAT-HRR-01</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>Punch-in</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr"/>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>Say how you are working when you punch in</t>
+        </is>
+      </c>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>1. Sign in as Ravi Engineer and open "Punch in / out".
+2. Under "Where are you working today?" choose "On duty" - a box "Where? (customer or place)" appears - type "Acme Forgings" and punch in.
+3. Next working day choose "Home" and punch in; on a third day leave "Office".</t>
+        </is>
+      </c>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
+          <t>- The choice is offered again next time (remembered, never forced); "On duty" asks where.
+- Today's card says how you are working (and the place); "My attendance" shows a "Worked as" column with Office / Home / On duty.</t>
+        </is>
+      </c>
+      <c r="H2" s="10" t="inlineStr"/>
+      <c r="I2" s="10" t="inlineStr"/>
+      <c r="J2" s="10" t="inlineStr"/>
+      <c r="K2" s="10" t="inlineStr"/>
+      <c r="L2" s="10" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>UAT-HRR-02</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Leave</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr"/>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>Apply for a half day and for a compensatory off</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>1. Open "My leave" &gt; "Apply for leave". Choose "Type of leave" = half day: only one date is asked and the dialog says "0.5 days of leave". Send it.
+2. Apply again with type compensatory off for a Saturday you worked: the dialog says it counts as 0 days of leave.</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>- Both requests appear in the list with their kind and days (0.5 and 0); Meera Manager sees the same on "Leave approvals" and can approve them.</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr"/>
+      <c r="I3" s="10" t="inlineStr"/>
+      <c r="J3" s="10" t="inlineStr"/>
+      <c r="K3" s="10" t="inlineStr"/>
+      <c r="L3" s="10" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>UAT-HRR-03</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Company settings</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr"/>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>Set the weekly off, late time and holidays</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>1. Open "Company settings" (Administration).
+2. Check the weekly off is Saturday + Sunday and the late time is 09:30; change the late time to 09:45, save.
+3. Add a holiday for tomorrow named "Founders day"; then remove it and confirm.</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>- Saving shows "Company settings saved."; the new holiday appears in the list; removing asks first, and the holiday disappears.
+- The Audit trail shows "Company settings changed", "Holiday added" and "Holiday removed".
+- Meera Manager (not the Owner) cannot open "Company settings".</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr"/>
+      <c r="I4" s="10" t="inlineStr"/>
+      <c r="J4" s="10" t="inlineStr"/>
+      <c r="K4" s="10" t="inlineStr"/>
+      <c r="L4" s="10" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>UAT-HRR-04</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr"/>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>The attendance analytics screen</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>1. Open "Attendance analytics" (Insights) as the Owner.
+2. Check the month tiles, "People working each day", "Where everyone's days went" and the per-employee table; click a column heading to sort.
+3. Change "Month" to last month and the "Financial year (leave)" to the previous one.</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>- Figures match what you know of the month (days worked, leave, late arrivals, absent days); lighter columns are weekly offs and holidays; "View as table" shows the same numbers.
+- The leave section shows days taken / still to come by month and per employee.</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr"/>
+      <c r="I5" s="10" t="inlineStr"/>
+      <c r="J5" s="10" t="inlineStr"/>
+      <c r="K5" s="10" t="inlineStr"/>
+      <c r="L5" s="10" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>UAT-HRR-05</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr"/>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>Download the four Excel reports and open them</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>1. On "Attendance analytics" use "Download as Excel (.xlsx)": pick Ravi Engineer and click "Monthly attendance", then "Leave card".
+2. Pick a day and click "Daily report"; click "Monthly summary (everyone)".
+3. Open each file in Excel / LibreOffice.</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>- Files are named like Attendance_Ravi_Engineer_October_2026.xlsx, LeaveCard_Ravi_Engineer.xlsx, DayReport_2026-10-14.xlsx and AttendanceSummary_October_2026.xlsx.
+- Each looks like the company's own sheet: a Type for every day (At Office, WFH, OD, WOW, HW, C/Off, W/Off, Holiday, FD Leave, HD Leave, Absent), colours, a legend and totals; the summary has a second "Day by day" sheet.
+- Half-day leave counts 0.5, comp-off 0; a remark such as =1+1 shows as text, never as a formula.</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr"/>
+      <c r="I6" s="10" t="inlineStr"/>
+      <c r="J6" s="10" t="inlineStr"/>
+      <c r="K6" s="10" t="inlineStr"/>
+      <c r="L6" s="10" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>UAT-HRR-06</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr"/>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Let the HR person download company reports</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>1. Create or choose a manager to act as HR (for example Meera Manager). As Meera, try to open Attendance analytics: it is refused and not in her menu.
+2. As the Owner open "Permissions" and grant Meera "Download company attendance reports" (global).
+3. As Meera reload and open "Attendance analytics"; download the daily report. Then, as the Owner, add a deny for Meera, and as Meera reload.</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>- Before the grant: "Not available" with an explanation; after: the screen opens, shows the WHOLE company (including Bharat's branch) and the downloads work; after the deny it closes again.
+- Meera's other screens still show only her own team.
+- The Audit trail records every "Report downloaded" with who and which report.</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr"/>
+      <c r="I7" s="10" t="inlineStr"/>
+      <c r="J7" s="10" t="inlineStr"/>
+      <c r="K7" s="10" t="inlineStr"/>
+      <c r="L7" s="10" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>UAT-HRR-07</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr"/>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>An employee cannot reach company reports</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>1. As Ravi Engineer type /attendance-analytics in the address bar.</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>- "Not available"; no figures and no downloads.</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr"/>
+      <c r="I8" s="10" t="inlineStr"/>
+      <c r="J8" s="10" t="inlineStr"/>
+      <c r="K8" s="10" t="inlineStr"/>
+      <c r="L8" s="10" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L8"/>
+  <conditionalFormatting sqref="I2:I8">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"Blocked"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="I2:I8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pass,Fail,Blocked,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6399,7 +6827,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>